<commit_message>
Restore rolling budget opening cash formulas
</commit_message>
<xml_diff>
--- a/vba/资金滚动预算模板.xlsx
+++ b/vba/资金滚动预算模板.xlsx
@@ -3437,12 +3437,24 @@
         <f>G39</f>
         <v>20000</v>
       </c>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="47"/>
+      <c r="I2" s="45">
+        <f>H39</f>
+      </c>
+      <c r="J2" s="45">
+        <f>I39</f>
+      </c>
+      <c r="K2" s="45">
+        <f>J39</f>
+      </c>
+      <c r="L2" s="45">
+        <f>K39</f>
+      </c>
+      <c r="M2" s="45">
+        <f>L39</f>
+      </c>
+      <c r="N2" s="47">
+        <f>M39</f>
+      </c>
       <c r="O2" s="36" t="s">
         <v>6</v>
       </c>

</xml_diff>